<commit_message>
#40 Improve details view.
</commit_message>
<xml_diff>
--- a/test/test-data/example_sp.xlsx
+++ b/test/test-data/example_sp.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\6svk\test\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8FC52D05-26E2-40A6-B4DB-CC9569749BFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2F5F040-10CC-462B-A17E-D256C10669A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="695" firstSheet="9" activeTab="9" xr2:uid="{73D0F693-E513-4638-BA68-582D5E75480A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="695" firstSheet="9" activeTab="9" xr2:uid="{73D0F693-E513-4638-BA68-582D5E75480A}"/>
   </bookViews>
   <sheets>
     <sheet name="MetaData" sheetId="14" r:id="rId1"/>
@@ -405,7 +405,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3581" uniqueCount="1678">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3792" uniqueCount="1683">
   <si>
     <r>
       <rPr>
@@ -6403,6 +6403,21 @@
   </si>
   <si>
     <t>Belegd in (onderzoeks)programma</t>
+  </si>
+  <si>
+    <t>SP_C2</t>
+  </si>
+  <si>
+    <t>SP_C1</t>
+  </si>
+  <si>
+    <t>Dit is een test programma waar het onderzoek mee te maken heeft.</t>
+  </si>
+  <si>
+    <t>In dit programma wordt het onderzoek belegd</t>
+  </si>
+  <si>
+    <t>Ook hier wordt een onderzoek belegd in een programma. Dit programma heeft een zeer lange naam en omschrijving, dus verwacht ik dat het over meerdere regels wordt weergegeven.</t>
   </si>
 </sst>
 </file>
@@ -14057,7 +14072,9 @@
         <f>"SP_"&amp;'Kennisagenda onderzoekslijnen'!C20</f>
         <v>SP_C1</v>
       </c>
-      <c r="C4" s="636"/>
+      <c r="C4" s="636" t="s">
+        <v>1678</v>
+      </c>
       <c r="D4" s="636"/>
       <c r="E4" s="147" t="str">
         <f>'Kennisagenda onderzoekslijnen'!F20</f>
@@ -14095,8 +14112,12 @@
         <f>'Kennisagenda onderzoekslijnen'!G20</f>
         <v>Technische levensduur - civiele delen</v>
       </c>
-      <c r="P4" s="666"/>
-      <c r="Q4" s="749"/>
+      <c r="P4" s="666" t="s">
+        <v>1680</v>
+      </c>
+      <c r="Q4" s="749" t="s">
+        <v>1681</v>
+      </c>
       <c r="R4" s="667"/>
       <c r="S4" s="662"/>
       <c r="T4" s="636"/>
@@ -14141,7 +14162,9 @@
         <f>"SP_"&amp;'Kennisagenda onderzoekslijnen'!C42</f>
         <v>SP_C2</v>
       </c>
-      <c r="C5" s="636"/>
+      <c r="C5" s="636" t="s">
+        <v>1679</v>
+      </c>
       <c r="D5" s="636"/>
       <c r="E5" s="707" t="str">
         <f>'Kennisagenda onderzoekslijnen'!F42</f>
@@ -14180,7 +14203,9 @@
         <v>Inspecties, monitoring en data</v>
       </c>
       <c r="P5" s="668"/>
-      <c r="Q5" s="750"/>
+      <c r="Q5" s="750" t="s">
+        <v>1682</v>
+      </c>
       <c r="R5" s="669"/>
       <c r="S5" s="662"/>
       <c r="T5" s="636"/>
@@ -19346,7 +19371,7 @@
     <mergeCell ref="Q1:Q2"/>
   </mergeCells>
   <phoneticPr fontId="28" type="noConversion"/>
-  <dataValidations disablePrompts="1" count="7">
+  <dataValidations count="7">
     <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="AG4:AG69" xr:uid="{81DA356F-6848-4732-B29B-4D9B463FEA67}">
       <formula1>"Duurzame leefomgeving,Droge voeten,Voldoende en schoon water, Vlot en veilig (weg en water),Betrouwbare en bruikbare informatie"</formula1>
     </dataValidation>

</xml_diff>